<commit_message>
Add Surveying tab with leads and sales from Airtable
</commit_message>
<xml_diff>
--- a/users/user-upload.xlsx
+++ b/users/user-upload.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markninnim/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markninnim/Documents/Claude/Projects/Digital Asset Management/users/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B33C2EDF-96C7-9D43-A613-C1ADA39A6D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC6A421-E0A0-5A48-8632-EFC791236A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,23 @@
     <sheet name="Upload Ready" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" refMode="R1C1" concurrentCalc="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Upload Ready'!$A$1:$O$119</definedName>
+  </definedNames>
+  <calcPr calcId="191029" refMode="R1C1" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1731,12 +1747,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:O119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="15" width="18" customWidth="1"/>
+    <col min="3" max="14" width="18" customWidth="1"/>
+    <col min="15" max="15" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -1786,7 +1804,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1821,7 +1839,7 @@
       </c>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -1856,7 +1874,7 @@
       </c>
       <c r="O3" s="2"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -1891,7 +1909,7 @@
       </c>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>29</v>
       </c>
@@ -1926,7 +1944,7 @@
       </c>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
@@ -1961,7 +1979,7 @@
       </c>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>37</v>
       </c>
@@ -1996,7 +2014,7 @@
       </c>
       <c r="O7" s="2"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>41</v>
       </c>
@@ -2031,7 +2049,7 @@
       </c>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>45</v>
       </c>
@@ -2063,7 +2081,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -2095,7 +2113,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -2127,7 +2145,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>57</v>
       </c>
@@ -2159,7 +2177,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>61</v>
       </c>
@@ -2191,7 +2209,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -2223,7 +2241,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>69</v>
       </c>
@@ -2252,7 +2270,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>72</v>
       </c>
@@ -2284,7 +2302,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>76</v>
       </c>
@@ -2316,7 +2334,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>80</v>
       </c>
@@ -2348,7 +2366,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>84</v>
       </c>
@@ -2380,7 +2398,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>88</v>
       </c>
@@ -2412,7 +2430,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>92</v>
       </c>
@@ -2444,7 +2462,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -2476,7 +2494,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>99</v>
       </c>
@@ -2508,7 +2526,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>102</v>
       </c>
@@ -2540,7 +2558,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>105</v>
       </c>
@@ -2572,7 +2590,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>108</v>
       </c>
@@ -2604,7 +2622,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>111</v>
       </c>
@@ -2636,7 +2654,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>115</v>
       </c>
@@ -2668,7 +2686,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>119</v>
       </c>
@@ -2700,7 +2718,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>123</v>
       </c>
@@ -2732,7 +2750,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>127</v>
       </c>
@@ -2764,7 +2782,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>131</v>
       </c>
@@ -2796,7 +2814,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>135</v>
       </c>
@@ -2828,7 +2846,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>139</v>
       </c>
@@ -2860,7 +2878,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>143</v>
       </c>
@@ -2892,7 +2910,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>143</v>
       </c>
@@ -2924,7 +2942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>135</v>
       </c>
@@ -2956,7 +2974,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>150</v>
       </c>
@@ -2988,7 +3006,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>154</v>
       </c>
@@ -3020,7 +3038,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>158</v>
       </c>
@@ -3052,7 +3070,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>135</v>
       </c>
@@ -3084,7 +3102,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>163</v>
       </c>
@@ -3116,7 +3134,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>167</v>
       </c>
@@ -3148,7 +3166,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>171</v>
       </c>
@@ -3180,7 +3198,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>175</v>
       </c>
@@ -3212,7 +3230,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>179</v>
       </c>
@@ -3244,7 +3262,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>183</v>
       </c>
@@ -3276,7 +3294,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>187</v>
       </c>
@@ -3308,7 +3326,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>135</v>
       </c>
@@ -3340,7 +3358,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>191</v>
       </c>
@@ -3372,7 +3390,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>195</v>
       </c>
@@ -3404,7 +3422,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -3436,7 +3454,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>202</v>
       </c>
@@ -3468,7 +3486,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>205</v>
       </c>
@@ -3500,7 +3518,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>209</v>
       </c>
@@ -3532,7 +3550,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>213</v>
       </c>
@@ -3564,7 +3582,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>217</v>
       </c>
@@ -3596,7 +3614,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>220</v>
       </c>
@@ -3628,7 +3646,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>224</v>
       </c>
@@ -3660,7 +3678,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>228</v>
       </c>
@@ -3692,7 +3710,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>231</v>
       </c>
@@ -3724,7 +3742,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>234</v>
       </c>
@@ -3756,7 +3774,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>238</v>
       </c>
@@ -3788,7 +3806,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>240</v>
       </c>
@@ -3820,7 +3838,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>242</v>
       </c>
@@ -3852,7 +3870,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>246</v>
       </c>
@@ -3884,7 +3902,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>249</v>
       </c>
@@ -3916,7 +3934,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>252</v>
       </c>
@@ -3948,7 +3966,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>255</v>
       </c>
@@ -3980,7 +3998,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>259</v>
       </c>
@@ -4012,7 +4030,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>261</v>
       </c>
@@ -4044,7 +4062,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>135</v>
       </c>
@@ -4076,7 +4094,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>266</v>
       </c>
@@ -4108,7 +4126,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>269</v>
       </c>
@@ -4140,7 +4158,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>272</v>
       </c>
@@ -4172,7 +4190,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>276</v>
       </c>
@@ -4204,7 +4222,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>279</v>
       </c>
@@ -4236,7 +4254,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>283</v>
       </c>
@@ -4268,7 +4286,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>287</v>
       </c>
@@ -4300,7 +4318,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>290</v>
       </c>
@@ -4332,7 +4350,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>294</v>
       </c>
@@ -4364,7 +4382,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>298</v>
       </c>
@@ -4396,7 +4414,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>301</v>
       </c>
@@ -4428,7 +4446,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>304</v>
       </c>
@@ -4460,7 +4478,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>308</v>
       </c>
@@ -4492,7 +4510,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>312</v>
       </c>
@@ -4524,7 +4542,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>316</v>
       </c>
@@ -4556,7 +4574,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>319</v>
       </c>
@@ -4588,7 +4606,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>323</v>
       </c>
@@ -4620,7 +4638,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>326</v>
       </c>
@@ -4652,7 +4670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>329</v>
       </c>
@@ -4684,7 +4702,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>333</v>
       </c>
@@ -4716,7 +4734,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>337</v>
       </c>
@@ -4748,7 +4766,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>340</v>
       </c>
@@ -4780,7 +4798,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>344</v>
       </c>
@@ -4812,7 +4830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>348</v>
       </c>
@@ -5324,7 +5342,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>405</v>
       </c>
@@ -5356,7 +5374,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>409</v>
       </c>
@@ -5388,7 +5406,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>412</v>
       </c>
@@ -5420,7 +5438,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>415</v>
       </c>
@@ -5452,7 +5470,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>417</v>
       </c>
@@ -5484,7 +5502,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>421</v>
       </c>
@@ -5516,7 +5534,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>425</v>
       </c>
@@ -5548,7 +5566,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:15" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>428</v>
       </c>
@@ -5581,6 +5599,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O119" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="14">
+      <filters>
+        <filter val="matt.stephens@financeplanning.co.uk"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>